<commit_message>
PAUSED (task136): rule 3 rework, stage 3 green, waiting on the reader and judge
Round 3: NPP-114's pooling clause and the prompt's binding removed; 4.1 files only the
impact at the design point. The decisive step is the bulk-buys' net addition, each past
campaign read against the suburbs whose campaign had not yet run. Call YRB27, 1.9 MW over
hosting capacity at 31 August 2029 (YRB24 1.7, gap 0.2; Bindarra Waters 1.7 MW, Wattleview
0.7 MW). Resume: stage 4, the leak reader and the determinism judge.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task136/golden/feeder_upgrade_2029.xlsx
+++ b/task136/golden/feeder_upgrade_2029.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="97">
   <si>
     <t>YRB27 takes the FY2027-28 hosting-capacity augmentation: its rooftop PV sits furthest above hosting capacity at the 31 August 2029 design point</t>
   </si>
@@ -55,19 +55,19 @@
     <t>Gap between them (MW)</t>
   </si>
   <si>
-    <t>Solar Streets 2026, Bindarra Waters (YRB24): PV added (MW)</t>
-  </si>
-  <si>
-    <t>Solar Streets 2026, Wattleview (YRB27): PV added (MW)</t>
-  </si>
-  <si>
-    <t>YRB27's rooftop PV is forecast at 25.2 MW on 31 August 2029 against a 2029 hosting capacity of 23.30 MW; 1.7 MW of it is the Wattleview bulk-buy.</t>
-  </si>
-  <si>
-    <t>Past Solar Streets campaigns installed about 1.17 systems for every first application their suburb's owner-occupied houses lodged in the year before sign-ups opened (505 systems on 431 applications over the seven campaigns). That is the only basis on which the seven agree; per home letterboxed or per house without PV they vary several-fold (Solar Streets sheet).</t>
-  </si>
-  <si>
-    <t>Wattleview's owner-occupiers lodged 209 first applications in the year to August 2026 and Bindarra Waters' lodged 52, so Wattleview's campaign is expected to add about four times as much PV although Bindarra Waters has more houses still without it.</t>
+    <t>Solar Streets 2026, Bindarra Waters (YRB24): PV added by 31 Aug 2029 (MW)</t>
+  </si>
+  <si>
+    <t>Solar Streets 2026, Wattleview (YRB27): PV added by 31 Aug 2029 (MW)</t>
+  </si>
+  <si>
+    <t>YRB27 forecast 16.1 MW at 31 Aug 2029 against 2029 hosting capacity 14.19 MW; 0.7 MW of it is the Wattleview bulk-buy.</t>
+  </si>
+  <si>
+    <t>Bulk-buys counted at what they add by the design point, not systems installed. The seven past campaigns installed 9.32 systems per 100 houses without PV, but more than half of those households would have gone solar within three years anyway; read against suburbs whose campaign had not yet run, they added 4.09 per 100 (Solar Streets tab).</t>
+  </si>
+  <si>
+    <t>Installed-systems basis puts YRB24 first. On the added basis Bindarra Waters (4,537 houses without PV) adds 1.7 MW and YRB24 stays 0.2 MW short of YRB27.</t>
   </si>
   <si>
     <t>Forecast rooftop PV (micro EG) at 31 August 2029 by feeder</t>
@@ -85,10 +85,10 @@
     <t>Base forecast 31 Aug 2029 (kW)</t>
   </si>
   <si>
-    <t>Solar Streets 2026 systems</t>
-  </si>
-  <si>
-    <t>Program capacity (kW)</t>
+    <t>Systems the 2026 bulk-buy adds</t>
+  </si>
+  <si>
+    <t>Bulk-buy addition (kW)</t>
   </si>
   <si>
     <t>Forecast 31 Aug 2029 (kW)</t>
@@ -124,10 +124,10 @@
     <t>Yarrabin</t>
   </si>
   <si>
-    <t>Connected capacity: each NMI's latest connected configuration on the network model's feeder; trend: the yearly increase in connected capacity less program systems first connected that year; program systems at the feeder's FY2025-26 average inverter rating (NPP-114 3.2, 4.1 to 4.3). Systems are carried unrounded.</t>
-  </si>
-  <si>
-    <t>Solar Streets: what a campaign installs, carried from the seven past campaigns</t>
+    <t>Connected capacity: each NMI's latest connected configuration on the network model's feeder. Trend: yearly increase in connected capacity less program systems first connected that year (NPP-114 3.2). Bulk-buy addition: systems the campaign adds by 31 Aug 2029 at the feeder's FY2025-26 average new inverter (4.1, 4.3). Carried unrounded.</t>
+  </si>
+  <si>
+    <t>Solar Streets: systems installed against systems added, seven past campaigns</t>
   </si>
   <si>
     <t>Campaign</t>
@@ -139,13 +139,31 @@
     <t>Sign-ups opened</t>
   </si>
   <si>
-    <t>First applications from owner-occupied houses, 12 months before sign-ups opened</t>
-  </si>
-  <si>
-    <t>Systems installed (program reference)</t>
-  </si>
-  <si>
-    <t>Systems per first application</t>
+    <t>Window to</t>
+  </si>
+  <si>
+    <t>Owner-occupied houses without PV at opening</t>
+  </si>
+  <si>
+    <t>Systems installed (program ref)</t>
+  </si>
+  <si>
+    <t>First applications, 12 months before</t>
+  </si>
+  <si>
+    <t>First applications in window (all, incl. program)</t>
+  </si>
+  <si>
+    <t>Comparison suburbs: window / 12 months before</t>
+  </si>
+  <si>
+    <t>Expected in window without campaign</t>
+  </si>
+  <si>
+    <t>Added by campaign</t>
+  </si>
+  <si>
+    <t>Added per 100 houses without PV</t>
   </si>
   <si>
     <t>GLM18</t>
@@ -193,31 +211,7 @@
     <t>All seven</t>
   </si>
   <si>
-    <t>Basis tried</t>
-  </si>
-  <si>
-    <t>Pooled rate over the seven</t>
-  </si>
-  <si>
-    <t>Lowest campaign</t>
-  </si>
-  <si>
-    <t>Highest campaign</t>
-  </si>
-  <si>
-    <t>Coefficient of variation</t>
-  </si>
-  <si>
-    <t>Per 100 homes letterboxed (the council's participation rate)</t>
-  </si>
-  <si>
-    <t>Per 100 owner-occupied houses in the suburb</t>
-  </si>
-  <si>
-    <t>Per 100 owner-occupied houses without PV when sign-ups opened</t>
-  </si>
-  <si>
-    <t>Per first application from the suburb's owner-occupied houses in the 12 months before sign-ups opened</t>
+    <t>Installed per 100 houses without PV, all seven: 9.32</t>
   </si>
   <si>
     <t>2026 campaign</t>
@@ -226,13 +220,13 @@
     <t>Sign-ups open</t>
   </si>
   <si>
-    <t>First applications from owner-occupied houses, 1 Sep 2025 to 31 Aug 2026</t>
-  </si>
-  <si>
-    <t>Systems added</t>
-  </si>
-  <si>
-    <t>Average inverter (kW, FY2025-26)</t>
+    <t>Owner-occupied houses without PV, 1 Sep 2026</t>
+  </si>
+  <si>
+    <t>Systems added by 31 Aug 2029</t>
+  </si>
+  <si>
+    <t>Average new inverter (kW, FY2025-26)</t>
   </si>
   <si>
     <t>PV added (MW)</t>
@@ -250,7 +244,7 @@
     <t>Wattleview</t>
   </si>
   <si>
-    <t>Owner-occupied house: rates roll land use 02 with rating R1, matched to NMIs through the GIS cross-reference. A first application is the earliest application at the NMI, other than a withdrawn one. Systems installed are the connected new systems lodged with the campaign's reference.</t>
+    <t>Owner-occupied house: rates roll land use 02, rating R1, matched to NMIs via the GIS cross-reference. First application: earliest application at the house other than a withdrawn one, by received date. Window: 36 months from sign-ups opening, or to 31 Aug 2026 for BNR23 and PBG24. Comparison: suburbs whose own campaign opens after the window (not yet treated). Expected without campaign = suburb's first applications in the 12 months before x comparison suburbs' window / 12-month ratio.</t>
   </si>
   <si>
     <t>Active DER Register sites by feeder, extract as at 31 August 2026</t>
@@ -310,7 +304,7 @@
     <t>Past campaigns</t>
   </si>
   <si>
-    <t>The council's Solar Streets summary, 2018 to 2024, for sign-up dates; systems counted from program references in the connection register, which agree with the council's systems installed for every campaign. The rate is pooled over the seven (clause 4.2).</t>
+    <t>Council Solar Streets summary 2018 to 2024 for sign-up dates; systems from program references in the connection register, which match the council's systems installed. What each campaign added is read against suburbs whose campaign had not yet run over the same months.</t>
   </si>
   <si>
     <t>DER Register</t>
@@ -329,10 +323,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="d mmm yyyy"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -422,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -444,8 +439,10 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -800,7 +797,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="4">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -808,7 +805,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="4">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -816,7 +813,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="4">
-        <v>0.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -824,7 +821,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="4">
-        <v>1.7</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -909,27 +906,27 @@
         <v>25</v>
       </c>
       <c r="B4" s="8">
-        <v>13600</v>
+        <v>18706</v>
       </c>
       <c r="C4" s="8">
-        <v>776</v>
+        <v>1098</v>
       </c>
       <c r="D4" s="8">
-        <v>15928</v>
+        <v>21998</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="8"/>
       <c r="G4" s="8">
-        <v>15928</v>
+        <v>21998</v>
       </c>
       <c r="H4" s="10">
-        <v>14.82</v>
+        <v>21.14</v>
       </c>
       <c r="I4" s="9">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="J4">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -937,24 +934,24 @@
         <v>26</v>
       </c>
       <c r="B5" s="8">
-        <v>20336</v>
+        <v>18531</v>
       </c>
       <c r="C5" s="8">
-        <v>1054</v>
+        <v>1551</v>
       </c>
       <c r="D5" s="8">
-        <v>23499</v>
+        <v>23185</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="8"/>
       <c r="G5" s="8">
-        <v>23499</v>
+        <v>23185</v>
       </c>
       <c r="H5" s="10">
-        <v>22.29</v>
+        <v>21.79</v>
       </c>
       <c r="I5" s="9">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="J5">
         <v>3</v>
@@ -965,21 +962,21 @@
         <v>27</v>
       </c>
       <c r="B6" s="8">
-        <v>10662</v>
+        <v>11954</v>
       </c>
       <c r="C6" s="8">
-        <v>498</v>
+        <v>810</v>
       </c>
       <c r="D6" s="8">
-        <v>12157</v>
+        <v>14385</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8">
-        <v>12157</v>
+        <v>14385</v>
       </c>
       <c r="H6" s="10">
-        <v>11.72</v>
+        <v>13.95</v>
       </c>
       <c r="I6" s="9">
         <v>0.4</v>
@@ -993,28 +990,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="8">
-        <v>4637</v>
+        <v>17845</v>
       </c>
       <c r="C7" s="8">
-        <v>498</v>
+        <v>1935</v>
       </c>
       <c r="D7" s="8">
-        <v>6130</v>
+        <v>23648</v>
       </c>
       <c r="E7" s="9">
-        <v>60.9</v>
+        <v>185.6</v>
       </c>
       <c r="F7" s="8">
-        <v>396</v>
+        <v>1698</v>
       </c>
       <c r="G7" s="8">
-        <v>6525</v>
+        <v>25346</v>
       </c>
       <c r="H7" s="10">
-        <v>5.13</v>
+        <v>23.65</v>
       </c>
       <c r="I7" s="9">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="J7">
         <v>2</v>
@@ -1025,27 +1022,27 @@
         <v>28</v>
       </c>
       <c r="B8" s="8">
-        <v>4733</v>
+        <v>21255</v>
       </c>
       <c r="C8" s="8">
-        <v>372</v>
+        <v>1736</v>
       </c>
       <c r="D8" s="8">
-        <v>5851</v>
+        <v>26462</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8">
-        <v>5851</v>
+        <v>26462</v>
       </c>
       <c r="H8" s="10">
-        <v>4.79</v>
+        <v>25.49</v>
       </c>
       <c r="I8" s="9">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -1053,21 +1050,21 @@
         <v>29</v>
       </c>
       <c r="B9" s="8">
-        <v>10370</v>
+        <v>11808</v>
       </c>
       <c r="C9" s="8">
-        <v>504</v>
+        <v>569</v>
       </c>
       <c r="D9" s="8">
-        <v>11884</v>
+        <v>13514</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8">
-        <v>11884</v>
+        <v>13514</v>
       </c>
       <c r="H9" s="10">
-        <v>12.54</v>
+        <v>14.17</v>
       </c>
       <c r="I9" s="9">
         <v>-0.7</v>
@@ -1081,25 +1078,25 @@
         <v>3</v>
       </c>
       <c r="B10" s="8">
-        <v>17938</v>
+        <v>11645</v>
       </c>
       <c r="C10" s="8">
-        <v>1852</v>
+        <v>1245</v>
       </c>
       <c r="D10" s="8">
-        <v>23495</v>
+        <v>15380</v>
       </c>
       <c r="E10" s="9">
-        <v>244.9</v>
+        <v>76</v>
       </c>
       <c r="F10" s="8">
-        <v>1707</v>
+        <v>710</v>
       </c>
       <c r="G10" s="8">
-        <v>25202</v>
+        <v>16090</v>
       </c>
       <c r="H10" s="10">
-        <v>23.3</v>
+        <v>14.19</v>
       </c>
       <c r="I10" s="9">
         <v>1.9</v>
@@ -1113,21 +1110,21 @@
         <v>30</v>
       </c>
       <c r="B11" s="8">
-        <v>10078</v>
+        <v>16554</v>
       </c>
       <c r="C11" s="8">
-        <v>540</v>
+        <v>1168</v>
       </c>
       <c r="D11" s="8">
-        <v>11698</v>
+        <v>20057</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="8"/>
       <c r="G11" s="8">
-        <v>11698</v>
+        <v>20057</v>
       </c>
       <c r="H11" s="10">
-        <v>10.99</v>
+        <v>19.34</v>
       </c>
       <c r="I11" s="9">
         <v>0.7</v>
@@ -1141,22 +1138,22 @@
         <v>31</v>
       </c>
       <c r="B12" s="12">
-        <v>92355</v>
+        <v>128297</v>
       </c>
       <c r="C12" s="12">
-        <v>6096</v>
+        <v>10111</v>
       </c>
       <c r="D12" s="12">
-        <v>110642</v>
+        <v>158629</v>
       </c>
       <c r="E12" s="13">
-        <v>305.8</v>
+        <v>261.5</v>
       </c>
       <c r="F12" s="12">
-        <v>2103</v>
+        <v>2408</v>
       </c>
       <c r="G12" s="12">
-        <v>112744</v>
+        <v>161037</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1172,25 +1169,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AD1995C-42C9-513D-861B-8743FF29CB14}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" customWidth="1"/>
-    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>34</v>
       </c>
@@ -1212,13 +1214,31 @@
       <c r="G3" s="7" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H3" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
         <v>25</v>
@@ -1226,22 +1246,40 @@
       <c r="D4" s="14">
         <v>43346</v>
       </c>
-      <c r="E4">
-        <v>16</v>
-      </c>
-      <c r="F4">
-        <v>19</v>
-      </c>
-      <c r="G4" s="10">
-        <v>1.19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E4" s="14">
+        <v>44441</v>
+      </c>
+      <c r="F4" s="8">
+        <v>1383</v>
+      </c>
+      <c r="G4" s="8">
+        <v>107</v>
+      </c>
+      <c r="H4" s="8">
+        <v>31</v>
+      </c>
+      <c r="I4" s="8">
+        <v>160</v>
+      </c>
+      <c r="J4" s="15">
+        <v>3.334</v>
+      </c>
+      <c r="K4" s="16">
+        <v>103.4</v>
+      </c>
+      <c r="L4" s="16">
+        <v>56.6</v>
+      </c>
+      <c r="M4" s="10">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
         <v>26</v>
@@ -1249,22 +1287,40 @@
       <c r="D5" s="14">
         <v>43710</v>
       </c>
-      <c r="E5">
-        <v>162</v>
-      </c>
-      <c r="F5">
+      <c r="E5" s="14">
+        <v>44805</v>
+      </c>
+      <c r="F5" s="8">
+        <v>2245</v>
+      </c>
+      <c r="G5" s="8">
         <v>180</v>
       </c>
-      <c r="G5" s="10">
-        <v>1.11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H5" s="8">
+        <v>57</v>
+      </c>
+      <c r="I5" s="8">
+        <v>281</v>
+      </c>
+      <c r="J5" s="15">
+        <v>3.404</v>
+      </c>
+      <c r="K5" s="16">
+        <v>194</v>
+      </c>
+      <c r="L5" s="16">
+        <v>87</v>
+      </c>
+      <c r="M5" s="10">
+        <v>3.87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
         <v>28</v>
@@ -1272,22 +1328,40 @@
       <c r="D6" s="14">
         <v>44445</v>
       </c>
-      <c r="E6">
-        <v>43</v>
-      </c>
-      <c r="F6">
+      <c r="E6" s="14">
+        <v>45540</v>
+      </c>
+      <c r="F6" s="8">
+        <v>5051</v>
+      </c>
+      <c r="G6" s="8">
+        <v>470</v>
+      </c>
+      <c r="H6" s="8">
+        <v>140</v>
+      </c>
+      <c r="I6" s="8">
+        <v>746</v>
+      </c>
+      <c r="J6" s="15">
+        <v>3.829</v>
+      </c>
+      <c r="K6" s="16">
+        <v>536</v>
+      </c>
+      <c r="L6" s="16">
+        <v>210</v>
+      </c>
+      <c r="M6" s="10">
+        <v>4.16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
         <v>53</v>
-      </c>
-      <c r="G6" s="10">
-        <v>1.23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" t="s">
-        <v>47</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -1295,22 +1369,40 @@
       <c r="D7" s="14">
         <v>44627</v>
       </c>
-      <c r="E7">
-        <v>81</v>
-      </c>
-      <c r="F7">
-        <v>109</v>
-      </c>
-      <c r="G7" s="10">
-        <v>1.35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E7" s="14">
+        <v>45722</v>
+      </c>
+      <c r="F7" s="8">
+        <v>1982</v>
+      </c>
+      <c r="G7" s="8">
+        <v>193</v>
+      </c>
+      <c r="H7" s="8">
+        <v>58</v>
+      </c>
+      <c r="I7" s="8">
+        <v>305</v>
+      </c>
+      <c r="J7" s="15">
+        <v>3.777</v>
+      </c>
+      <c r="K7" s="16">
+        <v>219.1</v>
+      </c>
+      <c r="L7" s="16">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="M7" s="10">
+        <v>4.34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -1318,22 +1410,40 @@
       <c r="D8" s="14">
         <v>44809</v>
       </c>
-      <c r="E8">
-        <v>41</v>
-      </c>
-      <c r="F8">
-        <v>48</v>
-      </c>
-      <c r="G8" s="10">
-        <v>1.17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E8" s="14">
+        <v>45904</v>
+      </c>
+      <c r="F8" s="8">
+        <v>1942</v>
+      </c>
+      <c r="G8" s="8">
+        <v>194</v>
+      </c>
+      <c r="H8" s="8">
+        <v>65</v>
+      </c>
+      <c r="I8" s="8">
+        <v>312</v>
+      </c>
+      <c r="J8" s="15">
+        <v>3.565</v>
+      </c>
+      <c r="K8" s="16">
+        <v>231.7</v>
+      </c>
+      <c r="L8" s="16">
+        <v>80.3</v>
+      </c>
+      <c r="M8" s="10">
+        <v>4.13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
         <v>29</v>
@@ -1341,22 +1451,40 @@
       <c r="D9" s="14">
         <v>45173</v>
       </c>
-      <c r="E9">
-        <v>33</v>
-      </c>
-      <c r="F9">
-        <v>34</v>
-      </c>
-      <c r="G9" s="10">
-        <v>1.03</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E9" s="14">
+        <v>46265</v>
+      </c>
+      <c r="F9" s="8">
+        <v>1414</v>
+      </c>
+      <c r="G9" s="8">
+        <v>140</v>
+      </c>
+      <c r="H9" s="8">
+        <v>56</v>
+      </c>
+      <c r="I9" s="8">
+        <v>229</v>
+      </c>
+      <c r="J9" s="15">
+        <v>3.137</v>
+      </c>
+      <c r="K9" s="16">
+        <v>175.6</v>
+      </c>
+      <c r="L9" s="16">
+        <v>53.4</v>
+      </c>
+      <c r="M9" s="10">
+        <v>3.77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
         <v>25</v>
@@ -1364,199 +1492,138 @@
       <c r="D10" s="14">
         <v>45537</v>
       </c>
-      <c r="E10">
-        <v>55</v>
-      </c>
-      <c r="F10">
+      <c r="E10" s="14">
+        <v>46265</v>
+      </c>
+      <c r="F10" s="8">
+        <v>1332</v>
+      </c>
+      <c r="G10" s="8">
+        <v>147</v>
+      </c>
+      <c r="H10" s="8">
+        <v>59</v>
+      </c>
+      <c r="I10" s="8">
+        <v>177</v>
+      </c>
+      <c r="J10" s="15">
+        <v>2.074</v>
+      </c>
+      <c r="K10" s="16">
+        <v>122.3</v>
+      </c>
+      <c r="L10" s="16">
+        <v>54.7</v>
+      </c>
+      <c r="M10" s="10">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="12">
+        <v>15349</v>
+      </c>
+      <c r="G11" s="12">
+        <v>1431</v>
+      </c>
+      <c r="L11" s="17">
+        <v>627.8</v>
+      </c>
+      <c r="M11" s="18">
+        <v>4.09</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="10">
-        <v>1.13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" s="11">
-        <v>431</v>
-      </c>
-      <c r="F11" s="11">
-        <v>505</v>
-      </c>
-      <c r="G11" s="15">
-        <v>1.172</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>60</v>
-      </c>
-      <c r="E14" s="10">
-        <v>1.94</v>
-      </c>
-      <c r="F14" s="10">
-        <v>0.6</v>
-      </c>
-      <c r="G14" s="10">
-        <v>4.38</v>
-      </c>
-      <c r="H14" s="10">
-        <v>0.72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" s="10">
-        <v>3.34</v>
-      </c>
-      <c r="F15" s="10">
-        <v>1.3</v>
-      </c>
-      <c r="G15" s="10">
-        <v>5.98</v>
+        <v>68</v>
+      </c>
+      <c r="B15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="14">
+        <v>46266</v>
+      </c>
+      <c r="F15" s="8">
+        <v>4537</v>
+      </c>
+      <c r="G15" s="9">
+        <v>185.6</v>
       </c>
       <c r="H15" s="10">
-        <v>0.61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>9.15</v>
+      </c>
+      <c r="I15" s="9">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" s="10">
-        <v>6.1</v>
-      </c>
-      <c r="F16" s="10">
-        <v>2.33</v>
-      </c>
-      <c r="G16" s="10">
-        <v>13.9</v>
+        <v>70</v>
+      </c>
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" s="14">
+        <v>46266</v>
+      </c>
+      <c r="F16" s="8">
+        <v>1857</v>
+      </c>
+      <c r="G16" s="9">
+        <v>76</v>
       </c>
       <c r="H16" s="10">
-        <v>0.71</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="16">
-        <v>1.172</v>
-      </c>
-      <c r="F17" s="16">
-        <v>1.03</v>
-      </c>
-      <c r="G17" s="16">
-        <v>1.346</v>
-      </c>
-      <c r="H17" s="10">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="58" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B20" t="s">
-        <v>71</v>
-      </c>
-      <c r="C20" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="14">
-        <v>46266</v>
-      </c>
-      <c r="E20">
-        <v>52</v>
-      </c>
-      <c r="F20" s="9">
-        <v>60.9</v>
-      </c>
-      <c r="G20" s="10">
-        <v>6.5</v>
-      </c>
-      <c r="H20" s="9">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+        <v>9.35</v>
+      </c>
+      <c r="I16" s="9">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="B21" t="s">
-        <v>73</v>
-      </c>
-      <c r="C21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" s="14">
-        <v>46266</v>
-      </c>
-      <c r="E21">
-        <v>209</v>
-      </c>
-      <c r="F21" s="9">
-        <v>244.9</v>
-      </c>
-      <c r="G21" s="10">
-        <v>6.97</v>
-      </c>
-      <c r="H21" s="9">
-        <v>1.7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1578,7 +1645,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="44" customHeight="1" x14ac:dyDescent="0.25">
@@ -1586,16 +1653,16 @@
         <v>15</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>77</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1603,16 +1670,16 @@
         <v>25</v>
       </c>
       <c r="B4" s="8">
-        <v>2323</v>
+        <v>3443</v>
       </c>
       <c r="C4" s="8">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="D4" s="8">
-        <v>14000</v>
+        <v>19280</v>
       </c>
       <c r="E4" s="8">
-        <v>1940</v>
+        <v>3260</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1620,16 +1687,16 @@
         <v>26</v>
       </c>
       <c r="B5" s="8">
-        <v>3448</v>
+        <v>3194</v>
       </c>
       <c r="C5" s="8">
-        <v>130</v>
+        <v>177</v>
       </c>
       <c r="D5" s="8">
-        <v>20680</v>
+        <v>18950</v>
       </c>
       <c r="E5" s="8">
-        <v>2410</v>
+        <v>2780</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1637,16 +1704,16 @@
         <v>27</v>
       </c>
       <c r="B6" s="8">
-        <v>1713</v>
+        <v>2128</v>
       </c>
       <c r="C6" s="8">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="D6" s="8">
-        <v>10860</v>
+        <v>12350</v>
       </c>
       <c r="E6" s="8">
-        <v>1310</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1654,16 +1721,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="8">
-        <v>702</v>
+        <v>2783</v>
       </c>
       <c r="C7" s="8">
-        <v>68</v>
+        <v>255</v>
       </c>
       <c r="D7" s="8">
-        <v>4730</v>
+        <v>18110</v>
       </c>
       <c r="E7" s="8">
-        <v>750</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1671,16 +1738,16 @@
         <v>28</v>
       </c>
       <c r="B8" s="8">
-        <v>717</v>
+        <v>3680</v>
       </c>
       <c r="C8" s="8">
-        <v>44</v>
+        <v>204</v>
       </c>
       <c r="D8" s="8">
-        <v>4850</v>
+        <v>21770</v>
       </c>
       <c r="E8" s="8">
-        <v>650</v>
+        <v>3080</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1688,16 +1755,16 @@
         <v>29</v>
       </c>
       <c r="B9" s="8">
-        <v>1996</v>
+        <v>2180</v>
       </c>
       <c r="C9" s="8">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="D9" s="8">
-        <v>10830</v>
+        <v>12200</v>
       </c>
       <c r="E9" s="8">
-        <v>1710</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1705,16 +1772,16 @@
         <v>3</v>
       </c>
       <c r="B10" s="8">
-        <v>2729</v>
+        <v>1838</v>
       </c>
       <c r="C10" s="8">
-        <v>252</v>
+        <v>158</v>
       </c>
       <c r="D10" s="8">
-        <v>18040</v>
+        <v>11800</v>
       </c>
       <c r="E10" s="8">
-        <v>2950</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1722,26 +1789,26 @@
         <v>30</v>
       </c>
       <c r="B11" s="8">
-        <v>1781</v>
+        <v>2927</v>
       </c>
       <c r="C11" s="8">
-        <v>62</v>
+        <v>159</v>
       </c>
       <c r="D11" s="8">
-        <v>10340</v>
+        <v>16980</v>
       </c>
       <c r="E11" s="8">
-        <v>1380</v>
+        <v>2510</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1760,71 +1827,71 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="20" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+    <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B4" s="20" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+    <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B5" s="20" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+    <row r="6" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B6" s="20" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B7" s="20" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
+    <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B8" s="20" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+    <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B9" s="20" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+    <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B10" s="20" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>